<commit_message>
Adjust Push scenario to land at €2M: 3 new AEs (Jul/Aug/Oct) instead of 4
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/work/WP_SEO_AI_Scenario_Planning.xlsx
+++ b/work/WP_SEO_AI_Scenario_Planning.xlsx
@@ -3084,7 +3084,7 @@
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
         <is>
-          <t>Deal cycle: 2 months (SQL → close). SQLs row shows when pipeline must be generated.</t>
+          <t>Deal cycle: 2 months (SQL → close). Pipeline row shows when SQLs must be generated.</t>
         </is>
       </c>
     </row>
@@ -3098,7 +3098,7 @@
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>Martijn: 0.6 FTE Apr-Jul, 0.5 FTE Aug+. Victor: 0.2→1.0 FTE (Jun for baseline/push, May for hyper-push).</t>
+          <t>Martijn: 0.6 FTE Apr-Jul, 0.5 FTE Aug+. Victor: 0.2→1.0 FTE (Jun baseline/push, May hyper-push).</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
     <row r="59">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>Hit €2M — hire ahead of pipeline</t>
+          <t>Hit €2M — staggered hiring, controlled acceleration</t>
         </is>
       </c>
     </row>
@@ -4292,21 +4292,21 @@
     <row r="62">
       <c r="A62" s="21" t="inlineStr">
         <is>
-          <t>We move faster: Victor full-time in June, two new AEs in July, a third in September. Martijn goes 0.5 FTE in August. BDR scales to 5 by Q4 with the SMB team contributing ~15 meetings/month on top. This gives us 4+ effective AEs by October — enough to run the full deal cadence across all three tiers.</t>
+          <t>The push scenario targets €2M new deal ARR with a measured ramp. Victor goes full-time in June. First new AE joins in July, a second in August, and a third in October — staggered to avoid overloading the pipeline and giving each hire time to absorb the narrative before the next one arrives. Martijn shifts to 0.5 FTE in August.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="21" t="inlineStr">
         <is>
-          <t>The bet: we can source and qualify enough MM pipeline to fill these seats. The dedicated BDR team needs to deliver 70 meetings/month by Q4, on top of the 15 from SMB spillover. That's 85 qualified MM meetings monthly. At 10% close rate, that's 8-9 deals/month closing by Q4.</t>
+          <t>BDR scales to 4 by Q3 and 5 by Q4, supplemented by ~15 MM meetings/month from the SMB team. By October we have 4+ effective AEs producing. The deal cadence compounds: Q4 alone delivers roughly 40% of the total ARR as the hiring investments from Q3 hit full productivity.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="21" t="inlineStr">
         <is>
-          <t>Risk profile: MEDIUM. Monthly burn peaks at €46K. We're hiring 4 new AEs before the first pilot cohort converts (Sep). If conversion disappoints, we're carrying cost against an unproven thesis. But if the motion works, push gets us to €2.4M new deal ARR and €2.5M total — well past the €2M target with room to overachieve.</t>
+          <t>Risk profile: MEDIUM. Monthly burn peaks at €38K. Three new AEs is a meaningful investment but not a bet-the-farm move. The staggered start gives us an exit ramp — if the first hire (July) underperforms by August, we can delay or redirect the October hire. If close rates hold at 10%, we land right at €2M. Expansion from pilot conversions adds upside toward €2.1M+.</t>
         </is>
       </c>
     </row>
@@ -4442,25 +4442,25 @@
         <v>0</v>
       </c>
       <c r="F69" s="25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G69" s="25" t="n">
         <v>2</v>
       </c>
       <c r="H69" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="I69" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J69" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="I69" s="25" t="n">
+      <c r="K69" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="J69" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="K69" s="25" t="n">
-        <v>4</v>
-      </c>
       <c r="L69" s="26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="70">
@@ -4491,37 +4491,37 @@
       </c>
       <c r="F70" s="27" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="G70" s="27" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.8</t>
         </is>
       </c>
       <c r="H70" s="27" t="inlineStr">
         <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="I70" s="27" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="J70" s="27" t="inlineStr">
+        <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="I70" s="27" t="inlineStr">
+      <c r="K70" s="27" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="J70" s="27" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="K70" s="27" t="inlineStr">
-        <is>
-          <t>5.2</t>
-        </is>
-      </c>
       <c r="L70" s="26" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
@@ -4590,7 +4590,7 @@
       </c>
       <c r="F72" s="27" t="inlineStr">
         <is>
-          <t>6.6</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="G72" s="27" t="inlineStr">
@@ -4600,22 +4600,22 @@
       </c>
       <c r="H72" s="27" t="inlineStr">
         <is>
+          <t>7.5</t>
+        </is>
+      </c>
+      <c r="I72" s="27" t="inlineStr">
+        <is>
           <t>8.5</t>
         </is>
       </c>
-      <c r="I72" s="27" t="inlineStr">
+      <c r="J72" s="27" t="inlineStr">
         <is>
           <t>9.5</t>
         </is>
       </c>
-      <c r="J72" s="27" t="inlineStr">
-        <is>
-          <t>10.5</t>
-        </is>
-      </c>
       <c r="K72" s="27" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="L72" s="26" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="F73" s="28" t="inlineStr">
         <is>
-          <t>€33.6k</t>
+          <t>€27.6k</t>
         </is>
       </c>
       <c r="G73" s="28" t="inlineStr">
@@ -4657,27 +4657,27 @@
       </c>
       <c r="H73" s="28" t="inlineStr">
         <is>
-          <t>€43.0k</t>
+          <t>€37.0k</t>
         </is>
       </c>
       <c r="I73" s="28" t="inlineStr">
         <is>
+          <t>€41.0k</t>
+        </is>
+      </c>
+      <c r="J73" s="28" t="inlineStr">
+        <is>
           <t>€47.0k</t>
         </is>
       </c>
-      <c r="J73" s="28" t="inlineStr">
-        <is>
-          <t>€53.0k</t>
-        </is>
-      </c>
       <c r="K73" s="28" t="inlineStr">
         <is>
-          <t>€53.0k</t>
+          <t>€47.0k</t>
         </is>
       </c>
       <c r="L73" s="26" t="inlineStr">
         <is>
-          <t>€299k total</t>
+          <t>€269k total</t>
         </is>
       </c>
     </row>
@@ -4772,25 +4772,25 @@
         <v>3</v>
       </c>
       <c r="F77" s="28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G77" s="28" t="n">
         <v>6</v>
       </c>
       <c r="H77" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="I77" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="J77" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="I77" s="28" t="n">
+      <c r="K77" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="J77" s="28" t="n">
-        <v>10</v>
-      </c>
-      <c r="K77" s="28" t="n">
-        <v>10</v>
-      </c>
       <c r="L77" s="26" t="n">
-        <v>54</v>
+        <v>46</v>
       </c>
     </row>
     <row r="78">
@@ -4817,7 +4817,7 @@
         <v>1</v>
       </c>
       <c r="G78" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H78" s="28" t="n">
         <v>2</v>
@@ -4829,10 +4829,10 @@
         <v>2</v>
       </c>
       <c r="K78" s="28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L78" s="26" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="79">
@@ -4868,13 +4868,13 @@
         <v>1</v>
       </c>
       <c r="J79" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K79" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L79" s="26" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80">
@@ -4893,25 +4893,25 @@
         <v>5</v>
       </c>
       <c r="F80" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G80" s="27" t="n">
+        <v>8</v>
+      </c>
+      <c r="H80" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="H80" s="27" t="n">
+      <c r="I80" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="J80" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="I80" s="27" t="n">
+      <c r="K80" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="J80" s="27" t="n">
-        <v>14</v>
-      </c>
-      <c r="K80" s="27" t="n">
-        <v>15</v>
-      </c>
       <c r="L80" s="26" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
     </row>
     <row r="82">
@@ -5025,25 +5025,25 @@
         <v>5</v>
       </c>
       <c r="H84" s="30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I84" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="J84" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="J84" s="30" t="n">
+      <c r="K84" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="L84" s="30" t="n">
         <v>11</v>
       </c>
-      <c r="K84" s="30" t="n">
+      <c r="M84" s="30" t="n">
         <v>11</v>
       </c>
-      <c r="L84" s="30" t="n">
-        <v>14</v>
-      </c>
-      <c r="M84" s="30" t="n">
-        <v>15</v>
-      </c>
       <c r="N84" s="29" t="n">
-        <v>76</v>
+        <v>64</v>
       </c>
     </row>
     <row r="85">
@@ -5067,23 +5067,23 @@
         <v>50</v>
       </c>
       <c r="F85" s="43" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G85" s="43" t="n">
+        <v>80</v>
+      </c>
+      <c r="H85" s="43" t="n">
         <v>90</v>
       </c>
-      <c r="H85" s="43" t="n">
+      <c r="I85" s="43" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" s="43" t="n">
         <v>110</v>
       </c>
-      <c r="I85" s="43" t="n">
+      <c r="K85" s="43" t="n">
         <v>110</v>
       </c>
-      <c r="J85" s="43" t="n">
-        <v>140</v>
-      </c>
-      <c r="K85" s="43" t="n">
-        <v>150</v>
-      </c>
       <c r="L85" s="43" t="inlineStr">
         <is>
           <t>-</t>
@@ -5095,7 +5095,7 @@
         </is>
       </c>
       <c r="N85" s="44" t="n">
-        <v>760</v>
+        <v>640</v>
       </c>
     </row>
     <row r="87">
@@ -5186,37 +5186,37 @@
       </c>
       <c r="F89" s="30" t="inlineStr">
         <is>
-          <t>€225k</t>
+          <t>€210k</t>
         </is>
       </c>
       <c r="G89" s="30" t="inlineStr">
         <is>
+          <t>€240k</t>
+        </is>
+      </c>
+      <c r="H89" s="30" t="inlineStr">
+        <is>
           <t>€290k</t>
         </is>
       </c>
-      <c r="H89" s="30" t="inlineStr">
+      <c r="I89" s="30" t="inlineStr">
+        <is>
+          <t>€305k</t>
+        </is>
+      </c>
+      <c r="J89" s="30" t="inlineStr">
         <is>
           <t>€320k</t>
         </is>
       </c>
-      <c r="I89" s="30" t="inlineStr">
+      <c r="K89" s="30" t="inlineStr">
         <is>
           <t>€320k</t>
         </is>
       </c>
-      <c r="J89" s="30" t="inlineStr">
-        <is>
-          <t>€450k</t>
-        </is>
-      </c>
-      <c r="K89" s="30" t="inlineStr">
-        <is>
-          <t>€500k</t>
-        </is>
-      </c>
       <c r="L89" s="29" t="inlineStr">
         <is>
-          <t>€2.36M</t>
+          <t>€1.94M</t>
         </is>
       </c>
     </row>
@@ -5230,54 +5230,54 @@
         <f> €2M target</f>
         <v/>
       </c>
-      <c r="C90" s="38" t="inlineStr">
+      <c r="C90" s="31" t="inlineStr">
         <is>
           <t>€30k</t>
         </is>
       </c>
-      <c r="D90" s="38" t="inlineStr">
+      <c r="D90" s="31" t="inlineStr">
         <is>
           <t>€60k</t>
         </is>
       </c>
-      <c r="E90" s="38" t="inlineStr">
+      <c r="E90" s="31" t="inlineStr">
         <is>
           <t>€255k</t>
         </is>
       </c>
-      <c r="F90" s="38" t="inlineStr">
-        <is>
-          <t>€480k</t>
-        </is>
-      </c>
-      <c r="G90" s="38" t="inlineStr">
-        <is>
-          <t>€770k</t>
-        </is>
-      </c>
-      <c r="H90" s="38" t="inlineStr">
-        <is>
-          <t>€1.09M</t>
-        </is>
-      </c>
-      <c r="I90" s="38" t="inlineStr">
-        <is>
-          <t>€1.41M</t>
-        </is>
-      </c>
-      <c r="J90" s="38" t="inlineStr">
-        <is>
-          <t>€1.86M</t>
-        </is>
-      </c>
-      <c r="K90" s="38" t="inlineStr">
-        <is>
-          <t>€2.36M</t>
-        </is>
-      </c>
-      <c r="L90" s="41" t="inlineStr">
-        <is>
-          <t>€2.36M</t>
+      <c r="F90" s="31" t="inlineStr">
+        <is>
+          <t>€465k</t>
+        </is>
+      </c>
+      <c r="G90" s="31" t="inlineStr">
+        <is>
+          <t>€705k</t>
+        </is>
+      </c>
+      <c r="H90" s="31" t="inlineStr">
+        <is>
+          <t>€995k</t>
+        </is>
+      </c>
+      <c r="I90" s="31" t="inlineStr">
+        <is>
+          <t>€1.30M</t>
+        </is>
+      </c>
+      <c r="J90" s="31" t="inlineStr">
+        <is>
+          <t>€1.62M</t>
+        </is>
+      </c>
+      <c r="K90" s="31" t="inlineStr">
+        <is>
+          <t>€1.94M</t>
+        </is>
+      </c>
+      <c r="L90" s="32" t="inlineStr">
+        <is>
+          <t>€1.94M</t>
         </is>
       </c>
     </row>
@@ -5366,37 +5366,37 @@
       </c>
       <c r="F92" s="35" t="inlineStr">
         <is>
-          <t>€480k</t>
+          <t>€465k</t>
         </is>
       </c>
       <c r="G92" s="35" t="inlineStr">
         <is>
-          <t>€770k</t>
+          <t>€705k</t>
         </is>
       </c>
       <c r="H92" s="35" t="inlineStr">
         <is>
-          <t>€1.12M</t>
+          <t>€1.03M</t>
         </is>
       </c>
       <c r="I92" s="35" t="inlineStr">
         <is>
-          <t>€1.48M</t>
+          <t>€1.37M</t>
         </is>
       </c>
       <c r="J92" s="35" t="inlineStr">
         <is>
-          <t>€1.97M</t>
+          <t>€1.73M</t>
         </is>
       </c>
       <c r="K92" s="35" t="inlineStr">
         <is>
-          <t>€2.54M</t>
+          <t>€2.12M</t>
         </is>
       </c>
       <c r="L92" s="36" t="inlineStr">
         <is>
-          <t>€2.54M</t>
+          <t>€2.12M</t>
         </is>
       </c>
     </row>
@@ -5410,20 +5410,20 @@
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>76 deals ÷ 10% = 760 meetings needed over 9 months</t>
+          <t>64 deals ÷ 10% = 640 meetings needed over 9 months</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="18">
-        <f> 85 meetings/month − 15 from SMB BDRs = 70 from dedicated BDRs</f>
+        <f> 72 meetings/month − 15 from SMB BDRs = 57 from dedicated BDRs</f>
         <v/>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="37" t="inlineStr">
         <is>
-          <t>70/mo ÷ 15/BDR = 5 dedicated MM BDRs needed</t>
+          <t>57/mo ÷ 15/BDR = 4 dedicated MM BDRs needed</t>
         </is>
       </c>
     </row>

</xml_diff>